<commit_message>
feat: persist super hide state to DB and misc updates
- Add super_hide to protocol (internal.fbs), DB user table, game character load/save
- Game server: character initial_params, to_protocol, login handler
- Internal server: Character model, repository, protocol wrapper and raw Character
- Regenerate FlatBuffer C++/C# for Character (super_hide)
- Update resources (maps.zip, door/map/mob/npc xlsx) and NPC scripts
- Include marriage.h, update_external.h, object_show.cpp changes
</commit_message>
<xml_diff>
--- a/resources/table/door.xlsx
+++ b/resources/table/door.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93BD1FF1-C720-4675-8223-E69084D9AD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB4D8A1-B881-45F8-A7DD-B80673CC6254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
   </bookViews>
   <sheets>
     <sheet name="door_pair" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
   <si>
     <t>open</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -239,6 +239,22 @@
   </si>
   <si>
     <t>[$door_pair]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>142 &amp; 143</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>63</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>144 &amp; 145</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>64</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -637,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C764A40-DCD2-43A8-BD02-A05E118C633D}">
-  <dimension ref="A1:C145"/>
+  <dimension ref="A1:C149"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9" style="1"/>
@@ -2238,6 +2254,50 @@
         <v>9804</v>
       </c>
     </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" s="1">
+        <v>142</v>
+      </c>
+      <c r="B146" s="1">
+        <v>4159</v>
+      </c>
+      <c r="C146" s="1">
+        <v>4161</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" s="1">
+        <v>143</v>
+      </c>
+      <c r="B147" s="1">
+        <v>4160</v>
+      </c>
+      <c r="C147" s="1">
+        <v>4162</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A148" s="1">
+        <v>144</v>
+      </c>
+      <c r="B148" s="1">
+        <v>4171</v>
+      </c>
+      <c r="C148" s="1">
+        <v>4173</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A149" s="1">
+        <v>145</v>
+      </c>
+      <c r="B149" s="1">
+        <v>4172</v>
+      </c>
+      <c r="C149" s="1">
+        <v>4174</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2246,7 +2306,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B8687D-3BEB-4B35-BC15-946421460DD0}">
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
@@ -2782,6 +2842,22 @@
         <v>62</v>
       </c>
     </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add on_spell_hit callback when spell target is hit
- Add object.on_spell_hit(from, spell) and mob Lua callback (on_spell_hit in model)
- Call to.on_spell_hit after life::active(spell, to) cast; rename fd to oid in life::active(spell, oid)
- Add mob model on_spell_hit field and regenerate model/Model.cs
- Fix map::movable hidden check to use x.hidden(object)
- Fix sky maze route display in command.lua (append secret slot 26)
- Add ON_MOB_SPELL_HIT to 백열장수련도우미 and 선풍각수련도우미 scripts
- Add effect, sound, action to 잠복근무 spell script
- Stat formatting and table resource updates (door, map, mob, npc)
</commit_message>
<xml_diff>
--- a/resources/table/door.xlsx
+++ b/resources/table/door.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB4D8A1-B881-45F8-A7DD-B80673CC6254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC95B082-28D7-4FFC-A015-4E502038CC81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
   <si>
     <t>open</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -255,6 +255,14 @@
   </si>
   <si>
     <t>64</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>146 &amp; 147</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>65</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -653,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C764A40-DCD2-43A8-BD02-A05E118C633D}">
-  <dimension ref="A1:C149"/>
+  <dimension ref="A1:C151"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9" style="1"/>
@@ -2298,6 +2306,28 @@
         <v>4174</v>
       </c>
     </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" s="1">
+        <v>146</v>
+      </c>
+      <c r="B150" s="1">
+        <v>8650</v>
+      </c>
+      <c r="C150" s="1">
+        <v>8674</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" s="1">
+        <v>147</v>
+      </c>
+      <c r="B151" s="1">
+        <v>8651</v>
+      </c>
+      <c r="C151" s="1">
+        <v>8675</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2306,7 +2336,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B8687D-3BEB-4B35-BC15-946421460DD0}">
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
@@ -2858,6 +2888,14 @@
         <v>67</v>
       </c>
     </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: log map block load failure instead of throwing
- Downgrade map block load failure from throw to warn in map_container::load
- Update door.xlsx and map.xlsx table data
</commit_message>
<xml_diff>
--- a/resources/table/door.xlsx
+++ b/resources/table/door.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC95B082-28D7-4FFC-A015-4E502038CC81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8E7560-338F-4233-A149-075A92D23C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
   </bookViews>
   <sheets>
     <sheet name="door_pair" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="79">
   <si>
     <t>open</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -263,6 +263,38 @@
   </si>
   <si>
     <t>65</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>148 &amp; 149</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>150 &amp; 151</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>152 &amp; 153 &amp; 154 &amp; 155</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>66</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>67</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>68</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>156 &amp; 157</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>69</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -661,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C764A40-DCD2-43A8-BD02-A05E118C633D}">
-  <dimension ref="A1:C151"/>
+  <dimension ref="A1:C161"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9" style="1"/>
@@ -2328,6 +2360,116 @@
         <v>8675</v>
       </c>
     </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" s="1">
+        <v>148</v>
+      </c>
+      <c r="B152" s="1">
+        <v>5572</v>
+      </c>
+      <c r="C152" s="1">
+        <v>5574</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" s="1">
+        <v>149</v>
+      </c>
+      <c r="B153" s="1">
+        <v>5573</v>
+      </c>
+      <c r="C153" s="1">
+        <v>5575</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" s="1">
+        <v>150</v>
+      </c>
+      <c r="B154" s="1">
+        <v>2875</v>
+      </c>
+      <c r="C154" s="1">
+        <v>2871</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" s="1">
+        <v>151</v>
+      </c>
+      <c r="B155" s="1">
+        <v>2876</v>
+      </c>
+      <c r="C155" s="1">
+        <v>2872</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" s="1">
+        <v>152</v>
+      </c>
+      <c r="B156" s="1">
+        <v>8627</v>
+      </c>
+      <c r="C156" s="1">
+        <v>8623</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A157" s="1">
+        <v>153</v>
+      </c>
+      <c r="B157" s="1">
+        <v>8628</v>
+      </c>
+      <c r="C157" s="1">
+        <v>8624</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A158" s="1">
+        <v>154</v>
+      </c>
+      <c r="B158" s="1">
+        <v>8629</v>
+      </c>
+      <c r="C158" s="1">
+        <v>8625</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" s="1">
+        <v>155</v>
+      </c>
+      <c r="B159" s="1">
+        <v>8630</v>
+      </c>
+      <c r="C159" s="1">
+        <v>8626</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160" s="1">
+        <v>156</v>
+      </c>
+      <c r="B160" s="1">
+        <v>265</v>
+      </c>
+      <c r="C160" s="1">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161" s="1">
+        <v>157</v>
+      </c>
+      <c r="B161" s="1">
+        <v>266</v>
+      </c>
+      <c r="C161" s="1">
+        <v>288</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2336,7 +2478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B8687D-3BEB-4B35-BC15-946421460DD0}">
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
@@ -2896,6 +3038,38 @@
         <v>69</v>
       </c>
     </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor: rename portrait to appearance and add mimicry support
- Rename portrait to appearance (headers, implementation, resources)
- Add mimicry protocol and generated code
- Update character, dialog, and external protocol
- Add appearance table, remove preset table
- Update builtin character, life, map, mob, model, npc
- Update Lua scripts (npc, item, spell, command, interaction)
- Update HTTP/FlatBuffer model and repository for mimicry
</commit_message>
<xml_diff>
--- a/resources/table/door.xlsx
+++ b/resources/table/door.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8E7560-338F-4233-A149-075A92D23C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0AECF46-8BD4-47D1-81B3-6965821209F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2DE58077-54AB-4A07-B369-A8F5921D9DEE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="81">
   <si>
     <t>open</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -295,6 +295,14 @@
   </si>
   <si>
     <t>69</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>70</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>158 &amp; 159</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -693,7 +701,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C764A40-DCD2-43A8-BD02-A05E118C633D}">
-  <dimension ref="A1:C161"/>
+  <dimension ref="A1:C163"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9" style="1"/>
@@ -2390,7 +2398,7 @@
         <v>2875</v>
       </c>
       <c r="C154" s="1">
-        <v>2871</v>
+        <v>2873</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
@@ -2401,7 +2409,7 @@
         <v>2876</v>
       </c>
       <c r="C155" s="1">
-        <v>2872</v>
+        <v>2874</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
@@ -2468,6 +2476,28 @@
       </c>
       <c r="C161" s="1">
         <v>288</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162" s="1">
+        <v>158</v>
+      </c>
+      <c r="B162" s="1">
+        <v>2885</v>
+      </c>
+      <c r="C162" s="1">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163" s="1">
+        <v>159</v>
+      </c>
+      <c r="B163" s="1">
+        <v>2886</v>
+      </c>
+      <c r="C163" s="1">
+        <v>2884</v>
       </c>
     </row>
   </sheetData>
@@ -2478,7 +2508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33B8687D-3BEB-4B35-BC15-946421460DD0}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
@@ -3070,6 +3100,14 @@
         <v>77</v>
       </c>
     </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>